<commit_message>
[tsomsomm] : [PowderShop] 리피파이 더미 컷신 추가
</commit_message>
<xml_diff>
--- a/data/_meta/LocalData.xlsx
+++ b/data/_meta/LocalData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -972,12 +972,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CutsceneData.CutsceneSelection.1000014</t>
+          <t>CutsceneData.Cutscene.1000033.1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>맞아</t>
+          <t>여긴 지솜님이 다음 빌드에 작업할거야.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -986,12 +986,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CutsceneData.CutsceneSelection.1000015</t>
+          <t>CutsceneData.CutsceneSelection.1000014</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>글쎄?</t>
+          <t>맞아</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1000,12 +1000,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000006</t>
+          <t>CutsceneData.CutsceneSelection.1000015</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>솔라리</t>
+          <t>글쎄?</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -1014,12 +1014,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000018</t>
+          <t>ItemData.Item.1000006</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>스틱</t>
+          <t>솔라리</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -1028,12 +1028,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000019</t>
+          <t>ItemData.Item.1000018</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>파우더</t>
+          <t>스틱</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -1042,12 +1042,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000020</t>
+          <t>ItemData.Item.1000019</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>버블건</t>
+          <t>파우더</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1056,12 +1056,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000021</t>
+          <t>ItemData.Item.1000020</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>그라인더</t>
+          <t>버블건</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1070,12 +1070,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000022</t>
+          <t>ItemData.Item.1000021</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>펜던트</t>
+          <t>그라인더</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1084,12 +1084,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000007</t>
+          <t>ItemData.Item.1000022</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>로딩 내용 어쩌고 저쩌고1</t>
+          <t>펜던트</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -1098,12 +1098,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000008</t>
+          <t>LoadingData.Loading.1000007</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>로딩 내용 어쩌고 저쩌고2</t>
+          <t>로딩 내용 어쩌고 저쩌고1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -1112,12 +1112,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000027</t>
+          <t>LoadingData.Loading.1000008</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>솜사탕상점 로딩화면</t>
+          <t>로딩 내용 어쩌고 저쩌고2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -1126,12 +1126,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000028</t>
+          <t>LoadingData.Loading.1000027</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>파우더상점 로딩화면</t>
+          <t>솜사탕상점 로딩화면</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -1140,12 +1140,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000029</t>
+          <t>LoadingData.Loading.1000028</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>이불상점 로딩화면</t>
+          <t>파우더상점 로딩화면</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -1154,12 +1154,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MapNpcData.MapNpcMenu.1000009.1</t>
+          <t>LoadingData.Loading.1000029</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>말걸기</t>
+          <t>이불상점 로딩화면</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -1168,12 +1168,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MapNpcData.MapNpcMenu.1000009.2</t>
+          <t>MapNpcData.MapNpcMenu.1000009.1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>미니게임 시작</t>
+          <t>말걸기</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -1182,12 +1182,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MapNpcData.MapNpcMenu.1000030.1</t>
+          <t>MapNpcData.MapNpcMenu.1000009.2</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>말걸기</t>
+          <t>미니게임 시작</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -1196,16 +1196,30 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MapNpcData.MapStaticNpcMenu.1000031.1</t>
+          <t>MapNpcData.MapNpcMenu.1000030.1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>미니게임 시작</t>
+          <t>말걸기</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>MapNpcData.MapStaticNpcMenu.1000031.1</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>미니게임 시작</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[tsomsomm] : 칼럼타입 수정
</commit_message>
<xml_diff>
--- a/data/_meta/LocalData.xlsx
+++ b/data/_meta/LocalData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D103"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -989,12 +989,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000006</t>
+          <t>EnumData.Enum.ItemType.1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>솔라리</t>
+          <t>솔라 화폐</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -1003,11 +1003,13 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000006.1</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>111</v>
+          <t>EnumData.Enum.ItemType.2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>마도구</t>
+        </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
@@ -1015,12 +1017,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000018</t>
+          <t>EnumData.Enum.ItemType.3</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>스틱</t>
+          <t>회복약</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -1029,11 +1031,13 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000018.1</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>222</v>
+          <t>EnumData.Enum.ItemType.4</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>사역마 회복약</t>
+        </is>
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
@@ -1041,12 +1045,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000019</t>
+          <t>EnumData.Enum.ItemType.5</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>파우더</t>
+          <t>사역마 지침 회복약</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1055,11 +1059,13 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000019.2</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>333</v>
+          <t>EnumData.Enum.ItemType.6</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>정제된 재료</t>
+        </is>
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
@@ -1067,12 +1073,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000020</t>
+          <t>EnumData.Enum.ItemType.7</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>버블건</t>
+          <t>재료</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -1081,11 +1087,13 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000020.3</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>444</v>
+          <t>EnumData.Enum.ItemType.8</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>퀘스트</t>
+        </is>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
@@ -1093,12 +1101,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000021</t>
+          <t>EnumData.Enum.ItemType.9</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>그라인더</t>
+          <t>탈 것</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -1107,11 +1115,13 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000021.4</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>555</v>
+          <t>EnumData.Enum.ItemType.10</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>사역마 소환</t>
+        </is>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
@@ -1119,12 +1129,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000022</t>
+          <t>ItemData.Item.1000006</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>펜던트</t>
+          <t>솔라리</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -1133,11 +1143,11 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000022.5</t>
+          <t>ItemData.Item.1000006.1</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>666</v>
+        <v>111</v>
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
@@ -1145,12 +1155,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000041</t>
+          <t>ItemData.Item.1000018</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>문라이트 베일 파우더</t>
+          <t>스틱</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -1159,11 +1169,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000041.6</t>
+          <t>ItemData.Item.1000018.1</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>32323</v>
+        <v>222</v>
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
@@ -1171,12 +1181,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000042</t>
+          <t>ItemData.Item.1000019</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>러브문 글로우 파우더</t>
+          <t>파우더</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
@@ -1185,11 +1195,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000042.7</t>
+          <t>ItemData.Item.1000019.2</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>43434</v>
+        <v>333</v>
       </c>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
@@ -1197,12 +1207,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000057</t>
+          <t>ItemData.Item.1000020</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>슈가 문 스틱</t>
+          <t>버블건</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -1211,13 +1221,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000036</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>하급 접착제</t>
-        </is>
+          <t>ItemData.Item.1000020.3</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>444</v>
       </c>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
@@ -1225,11 +1233,13 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000036.1</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>777</v>
+          <t>ItemData.Item.1000021</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>그라인더</t>
+        </is>
       </c>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
@@ -1237,13 +1247,11 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000037</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>중급 접착제</t>
-        </is>
+          <t>ItemData.Item.1000021.4</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>555</v>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
@@ -1251,11 +1259,13 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000037.2</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>888</v>
+          <t>ItemData.Item.1000022</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>펜던트</t>
+        </is>
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
@@ -1263,13 +1273,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000038</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">고급 접착제 </t>
-        </is>
+          <t>ItemData.Item.1000022.5</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>666</v>
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr"/>
@@ -1277,11 +1285,13 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000038.3</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>999</v>
+          <t>ItemData.Item.1000041</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>문라이트 베일 파우더</t>
+        </is>
       </c>
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr"/>
@@ -1289,13 +1299,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000039</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>최고급 접착제</t>
-        </is>
+          <t>ItemData.Item.1000041.6</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>32323</v>
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr"/>
@@ -1303,12 +1311,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000058</t>
+          <t>ItemData.Item.1000042</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>오로라 파르페</t>
+          <t>러브문 글로우 파우더</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -1317,13 +1325,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000058.5</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>오로라 파르페</t>
-        </is>
+          <t>ItemData.Item.1000042.7</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>43434</v>
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
@@ -1331,12 +1337,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000059</t>
+          <t>ItemData.Item.1000057</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>미카의 포토카드</t>
+          <t>슈가 문 스틱</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -1345,12 +1351,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000059.6</t>
+          <t>ItemData.Item.1000036</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>미카의 포토카드</t>
+          <t>하급 접착제</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -1359,13 +1365,11 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000060</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>농땡이 파우더 캐슬</t>
-        </is>
+          <t>ItemData.Item.1000036.1</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>777</v>
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr"/>
@@ -1373,12 +1377,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000060.7</t>
+          <t>ItemData.Item.1000037</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>농땡이 파우더 캐슬</t>
+          <t>중급 접착제</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -1387,13 +1391,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000046</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>파우더 가루</t>
-        </is>
+          <t>ItemData.Item.1000037.2</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>888</v>
       </c>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr"/>
@@ -1401,12 +1403,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000046.8</t>
+          <t>ItemData.Item.1000038</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>파우더 가루</t>
+          <t xml:space="preserve">고급 접착제 </t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -1415,13 +1417,11 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000043</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>리피파이 수제 파우더</t>
-        </is>
+          <t>ItemData.Item.1000038.3</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>999</v>
       </c>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr"/>
@@ -1429,12 +1429,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000043.1</t>
+          <t>ItemData.Item.1000039</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>리피파이 수제 파우더</t>
+          <t>최고급 접착제</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -1443,12 +1443,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000044</t>
+          <t>ItemData.Item.1000058</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>더스트 펄</t>
+          <t>오로라 파르페</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -1457,12 +1457,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000044.1</t>
+          <t>ItemData.Item.1000058.5</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>더스트 펄</t>
+          <t>오로라 파르페</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
@@ -1471,12 +1471,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000061</t>
+          <t>ItemData.Item.1000059</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>폭신폭신 사역마 쿠션</t>
+          <t>미카의 포토카드</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -1485,12 +1485,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000061.2</t>
+          <t>ItemData.Item.1000059.6</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>폭신폭신 사역마 쿠션</t>
+          <t>미카의 포토카드</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -1499,12 +1499,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000062</t>
+          <t>ItemData.Item.1000060</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>부숭부숭 사역마 목도리</t>
+          <t>농땡이 파우더 캐슬</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -1513,12 +1513,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000062.3</t>
+          <t>ItemData.Item.1000060.7</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>부숭부숭 사역마 목도리</t>
+          <t>농땡이 파우더 캐슬</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -1527,12 +1527,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000063</t>
+          <t>ItemData.Item.1000046</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>실키 클라우드 퍼프</t>
+          <t>파우더 가루</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
@@ -1541,12 +1541,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000063.1</t>
+          <t>ItemData.Item.1000046.8</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>실키 클라우드 퍼프</t>
+          <t>파우더 가루</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -1555,12 +1555,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000045</t>
+          <t>ItemData.Item.1000043</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>노랑 파우더 가루</t>
+          <t>리피파이 수제 파우더</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -1569,12 +1569,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000045.1</t>
+          <t>ItemData.Item.1000043.1</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>노랑 파우더 가루</t>
+          <t>리피파이 수제 파우더</t>
         </is>
       </c>
       <c r="C83" t="inlineStr"/>
@@ -1583,12 +1583,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000064</t>
+          <t>ItemData.Item.1000044</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>솜솜가루</t>
+          <t>더스트 펄</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -1597,12 +1597,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000064.2</t>
+          <t>ItemData.Item.1000044.1</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>솜솜가루</t>
+          <t>더스트 펄</t>
         </is>
       </c>
       <c r="C85" t="inlineStr"/>
@@ -1611,12 +1611,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000065</t>
+          <t>ItemData.Item.1000061</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>솜뭉치 씨앗</t>
+          <t>폭신폭신 사역마 쿠션</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
@@ -1625,12 +1625,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000065.3</t>
+          <t>ItemData.Item.1000061.2</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>솜뭉치 씨앗</t>
+          <t>폭신폭신 사역마 쿠션</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
@@ -1639,12 +1639,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000066</t>
+          <t>ItemData.Item.1000062</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>바삭바삭 꿈뭉치</t>
+          <t>부숭부숭 사역마 목도리</t>
         </is>
       </c>
       <c r="C88" t="inlineStr"/>
@@ -1653,12 +1653,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000066.4</t>
+          <t>ItemData.Item.1000062.3</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>바삭바삭 꿈뭉치</t>
+          <t>부숭부숭 사역마 목도리</t>
         </is>
       </c>
       <c r="C89" t="inlineStr"/>
@@ -1667,12 +1667,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000067</t>
+          <t>ItemData.Item.1000063</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>솜사탕</t>
+          <t>실키 클라우드 퍼프</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
@@ -1681,12 +1681,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000067.1</t>
+          <t>ItemData.Item.1000063.1</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>솜사탕</t>
+          <t>실키 클라우드 퍼프</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -1695,12 +1695,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000068</t>
+          <t>ItemData.Item.1000045</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>페로페로 향수</t>
+          <t>노랑 파우더 가루</t>
         </is>
       </c>
       <c r="C92" t="inlineStr"/>
@@ -1709,12 +1709,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000068.1</t>
+          <t>ItemData.Item.1000045.1</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>페로페로 향수</t>
+          <t>노랑 파우더 가루</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -1723,12 +1723,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000069</t>
+          <t>ItemData.Item.1000064</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>솜솜 보틀</t>
+          <t>솜솜가루</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -1737,12 +1737,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000069.1</t>
+          <t>ItemData.Item.1000064.2</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>솜솜 보틀</t>
+          <t>솜솜가루</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -1751,12 +1751,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000007</t>
+          <t>ItemData.Item.1000065</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>로딩 내용 어쩌고 저쩌고1</t>
+          <t>솜뭉치 씨앗</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -1765,12 +1765,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000008</t>
+          <t>ItemData.Item.1000065.3</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>로딩 내용 어쩌고 저쩌고2</t>
+          <t>솜뭉치 씨앗</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -1779,12 +1779,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000027</t>
+          <t>ItemData.Item.1000066</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>솜사탕상점 로딩화면</t>
+          <t>바삭바삭 꿈뭉치</t>
         </is>
       </c>
       <c r="C98" t="inlineStr"/>
@@ -1793,12 +1793,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000028</t>
+          <t>ItemData.Item.1000066.4</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>파우더상점 로딩화면</t>
+          <t>바삭바삭 꿈뭉치</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -1807,12 +1807,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000029</t>
+          <t>ItemData.Item.1000067</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>이불상점 로딩화면</t>
+          <t>솜사탕</t>
         </is>
       </c>
       <c r="C100" t="inlineStr"/>
@@ -1821,12 +1821,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MapNpcData.MapNpcMenu.1000009.1</t>
+          <t>ItemData.Item.1000067.1</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>미니게임 시작</t>
+          <t>솜사탕</t>
         </is>
       </c>
       <c r="C101" t="inlineStr"/>
@@ -1835,12 +1835,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>MapNpcData.MapNpcMenu.1000030.1</t>
+          <t>ItemData.Item.1000068</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>말걸기</t>
+          <t>페로페로 향수</t>
         </is>
       </c>
       <c r="C102" t="inlineStr"/>
@@ -1849,16 +1849,156 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MapNpcData.MapStaticNpcMenu.1000031.1</t>
+          <t>ItemData.Item.1000068.1</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>미니게임 시작</t>
+          <t>페로페로 향수</t>
         </is>
       </c>
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>ItemData.Item.1000069</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>솜솜 보틀</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>ItemData.Item.1000069.1</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>솜솜 보틀</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>LoadingData.Loading.1000007</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>로딩 내용 어쩌고 저쩌고1</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>LoadingData.Loading.1000008</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>로딩 내용 어쩌고 저쩌고2</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>LoadingData.Loading.1000027</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>솜사탕상점 로딩화면</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>LoadingData.Loading.1000028</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>파우더상점 로딩화면</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr"/>
+      <c r="D109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>LoadingData.Loading.1000029</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>이불상점 로딩화면</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>MapNpcData.MapNpcMenu.1000009.1</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>미니게임 시작</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>MapNpcData.MapNpcMenu.1000030.1</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>말걸기</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>MapNpcData.MapStaticNpcMenu.1000031.1</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>미니게임 시작</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[tsomsomm] : 솜사탕 npc 데이터 추가
</commit_message>
<xml_diff>
--- a/data/_meta/LocalData.xlsx
+++ b/data/_meta/LocalData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D117"/>
+  <dimension ref="A1:D118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2070,6 +2070,20 @@
       <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr"/>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>MapNpcData.MapStaticNpcMenu.1000081.1</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>미니게임 시작</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr"/>
+      <c r="D118" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[tsomsomm] : 아티팩트 enum name 추가
</commit_message>
<xml_diff>
--- a/data/_meta/LocalData.xlsx
+++ b/data/_meta/LocalData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D119"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1171,12 +1171,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000006</t>
+          <t>EnumData.Enum.ArtifactType.1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>솔라리</t>
+          <t>스틱</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -1185,11 +1185,13 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000006.1</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>111</v>
+          <t>EnumData.Enum.ArtifactType.2</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>파우더</t>
+        </is>
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
@@ -1197,12 +1199,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000018</t>
+          <t>EnumData.Enum.ArtifactType.3</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>스틱</t>
+          <t>버블건</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -1211,12 +1213,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000018.1</t>
+          <t>EnumData.Enum.ArtifactType.4</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>초보 마법소녀 새턴이 「마법소녀 위클리」에서 주문한  '소녀의 꿈, 핑크 아티팩트 3종 세트'의 첫 번째 마도구. 빛나는 토성은 소녀에게 무엇을 보여주게 될까?</t>
+          <t>그라인더</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -1225,12 +1227,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000019</t>
+          <t>EnumData.Enum.ArtifactType.5</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>파우더</t>
+          <t>펜던트</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -1239,12 +1241,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000019.2</t>
+          <t>ItemData.Item.1000006</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>초보 마법소녀 새턴이 「마법소녀 위클리」에서 주문한  '소녀의 꿈, 핑크 아티팩트 3종 세트'의 두 번째 마도구. 7색의 보석은 소녀에게 어떤 꿈을 꾸게 해줄까?</t>
+          <t>솔라리</t>
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
@@ -1253,13 +1255,11 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000020</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>버블건</t>
-        </is>
+          <t>ItemData.Item.1000006.1</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>111</v>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
@@ -1267,12 +1267,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000020.3</t>
+          <t>ItemData.Item.1000018</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>초보 마법소녀 새턴이 「마법소녀 위클리」에서 주문한  '소녀의 꿈, 핑크 아티팩트 3종 세트'의 세 번째 마도구. 날개 달린 버블건은 소녀를 어디로 데려가줄까?</t>
+          <t>스틱</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -1281,12 +1281,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000021</t>
+          <t>ItemData.Item.1000018.1</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>그라인더</t>
+          <t>초보 마법소녀 새턴이 「마법소녀 위클리」에서 주문한  '소녀의 꿈, 핑크 아티팩트 3종 세트'의 첫 번째 마도구. 빛나는 토성은 소녀에게 무엇을 보여주게 될까?</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -1295,12 +1295,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000021.4</t>
+          <t>ItemData.Item.1000019</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>「마법소녀 위클리」에서 주문할 수 있는  '소녀의 꿈, 핑크 아티팩트 추가 2종 세트'의 마도구. 무엇이든 갈고, 섞고, 흩뿌려보자!</t>
+          <t>파우더</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -1309,12 +1309,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000022</t>
+          <t>ItemData.Item.1000019.2</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>펜던트</t>
+          <t>초보 마법소녀 새턴이 「마법소녀 위클리」에서 주문한  '소녀의 꿈, 핑크 아티팩트 3종 세트'의 두 번째 마도구. 7색의 보석은 소녀에게 어떤 꿈을 꾸게 해줄까?</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -1323,12 +1323,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000022.5</t>
+          <t>ItemData.Item.1000020</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>「마법소녀 위클리」에서 주문할 수 있는  '소녀의 꿈, 핑크 아티팩트 추가 2종 세트'의 마도구. 작지만 단단한 결정이 오래된 소망을 간직하고 있다.</t>
+          <t>버블건</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -1337,12 +1337,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000041</t>
+          <t>ItemData.Item.1000020.3</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>문라이트 베일 파우더</t>
+          <t>초보 마법소녀 새턴이 「마법소녀 위클리」에서 주문한  '소녀의 꿈, 핑크 아티팩트 3종 세트'의 세 번째 마도구. 날개 달린 버블건은 소녀를 어디로 데려가줄까?</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -1351,12 +1351,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000041.6</t>
+          <t>ItemData.Item.1000021</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>아무도 보지 않는 밤, 문라이트 베일 파우더는 더 밝게 빛을 발한다. 무엇으로든 변하고 싶은 마음은 소녀의 힘에 날개를 달아줄 것이다!</t>
+          <t>그라인더</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -1365,12 +1365,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000042</t>
+          <t>ItemData.Item.1000021.4</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>러브문 글로우 파우더</t>
+          <t>「마법소녀 위클리」에서 주문할 수 있는  '소녀의 꿈, 핑크 아티팩트 추가 2종 세트'의 마도구. 무엇이든 갈고, 섞고, 흩뿌려보자!</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -1379,12 +1379,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000042.7</t>
+          <t>ItemData.Item.1000022</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>러브문 글로우 파우더가 마법소녀에게 힘을 더한다. 사랑에 빠진 소녀의 열정을 막을 수 있는 건 아무것도 없지!</t>
+          <t>펜던트</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
@@ -1393,12 +1393,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000057</t>
+          <t>ItemData.Item.1000022.5</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>슈가 문 스틱</t>
+          <t>「마법소녀 위클리」에서 주문할 수 있는  '소녀의 꿈, 핑크 아티팩트 추가 2종 세트'의 마도구. 작지만 단단한 결정이 오래된 소망을 간직하고 있다.</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -1407,12 +1407,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000057.8</t>
+          <t>ItemData.Item.1000041</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>달빛보다 신비롭고 솜사탕보다 달콤한 마법소녀가 당신의 꿈이었다면!</t>
+          <t>문라이트 베일 파우더</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -1421,12 +1421,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000036</t>
+          <t>ItemData.Item.1000041.6</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>하급 접착제</t>
+          <t>아무도 보지 않는 밤, 문라이트 베일 파우더는 더 밝게 빛을 발한다. 무엇으로든 변하고 싶은 마음은 소녀의 힘에 날개를 달아줄 것이다!</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -1435,11 +1435,13 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000036.1</t>
-        </is>
-      </c>
-      <c r="B72" t="n">
-        <v>777</v>
+          <t>ItemData.Item.1000042</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>러브문 글로우 파우더</t>
+        </is>
       </c>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr"/>
@@ -1447,12 +1449,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000037</t>
+          <t>ItemData.Item.1000042.7</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>중급 접착제</t>
+          <t>러브문 글로우 파우더가 마법소녀에게 힘을 더한다. 사랑에 빠진 소녀의 열정을 막을 수 있는 건 아무것도 없지!</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -1461,11 +1463,13 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000037.2</t>
-        </is>
-      </c>
-      <c r="B74" t="n">
-        <v>888</v>
+          <t>ItemData.Item.1000057</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>슈가 문 스틱</t>
+        </is>
       </c>
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr"/>
@@ -1473,12 +1477,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000038</t>
+          <t>ItemData.Item.1000057.8</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">고급 접착제 </t>
+          <t>달빛보다 신비롭고 솜사탕보다 달콤한 마법소녀가 당신의 꿈이었다면!</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
@@ -1487,11 +1491,13 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000038.3</t>
-        </is>
-      </c>
-      <c r="B76" t="n">
-        <v>999</v>
+          <t>ItemData.Item.1000036</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>하급 접착제</t>
+        </is>
       </c>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr"/>
@@ -1499,13 +1505,11 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000039</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>최고급 접착제</t>
-        </is>
+          <t>ItemData.Item.1000036.1</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>777</v>
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr"/>
@@ -1513,12 +1517,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000058</t>
+          <t>ItemData.Item.1000037</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>미카의 오로라 파르페</t>
+          <t>중급 접착제</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -1527,13 +1531,11 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000058.5</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>솜사탕 가게의 숨겨진 메뉴로 미카의 기분이 내킬 때만 맛볼 수 있는 특제 오로라 파르페. 톡톡 튀는 팝핑캔디와 갖가지 캔디시럽이 내키는 대로 뒤섞인 아름다운 카오스가 황홀경을 맛보여준다고.</t>
-        </is>
+          <t>ItemData.Item.1000037.2</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>888</v>
       </c>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr"/>
@@ -1541,12 +1543,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000059</t>
+          <t>ItemData.Item.1000038</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>미카의 포토카드</t>
+          <t xml:space="preserve">고급 접착제 </t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
@@ -1555,13 +1557,11 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000059.6</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>아이돌 그룹의 멤버로 활동하던 시절에 소량 제작되었던 미카의 포토카드. 더이상 판매되지 않는 레어템이라 미카의 팬에게는 굉장한 보물일지도?!</t>
-        </is>
+          <t>ItemData.Item.1000038.3</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>999</v>
       </c>
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr"/>
@@ -1569,12 +1569,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000060</t>
+          <t>ItemData.Item.1000039</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>리피파이의 파우더리 캐슬</t>
+          <t>최고급 접착제</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -1583,12 +1583,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000060.7</t>
+          <t>ItemData.Item.1000058</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>리피파이의 손길이 구석구석 닿은 파우더 공예품. 본인은 그저 심심풀이로 만든 잡동사니라지만, 놀라운 섬세함이 눈길을 사로잡는다.</t>
+          <t>미카의 오로라 파르페</t>
         </is>
       </c>
       <c r="C83" t="inlineStr"/>
@@ -1597,12 +1597,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000046</t>
+          <t>ItemData.Item.1000058.5</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>파우더 가루</t>
+          <t>솜사탕 가게의 숨겨진 메뉴로 미카의 기분이 내킬 때만 맛볼 수 있는 특제 오로라 파르페. 톡톡 튀는 팝핑캔디와 갖가지 캔디시럽이 내키는 대로 뒤섞인 아름다운 카오스가 황홀경을 맛보여준다고.</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -1611,12 +1611,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000046.8</t>
+          <t>ItemData.Item.1000059</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>파우더 가루</t>
+          <t>미카의 포토카드</t>
         </is>
       </c>
       <c r="C85" t="inlineStr"/>
@@ -1625,12 +1625,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000043</t>
+          <t>ItemData.Item.1000059.6</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>뽀송 프로그 데오도란트</t>
+          <t>아이돌 그룹의 멤버로 활동하던 시절에 소량 제작되었던 미카의 포토카드. 더이상 판매되지 않는 레어템이라 미카의 팬에게는 굉장한 보물일지도?!</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
@@ -1639,12 +1639,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000043.1</t>
+          <t>ItemData.Item.1000060</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>이마에 맺힌 땀방울을 확실하게 잡아주는 뽀송 프로그 데오도란트. 기분 좋은 쿨링 효과가 체력을 50 회복시켜준다.</t>
+          <t>리피파이의 파우더리 캐슬</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
@@ -1653,12 +1653,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000044</t>
+          <t>ItemData.Item.1000060.7</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>더스트 펄</t>
+          <t>리피파이의 손길이 구석구석 닿은 파우더 공예품. 본인은 그저 심심풀이로 만든 잡동사니라지만, 놀라운 섬세함이 눈길을 사로잡는다.</t>
         </is>
       </c>
       <c r="C88" t="inlineStr"/>
@@ -1667,12 +1667,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000044.1</t>
+          <t>ItemData.Item.1000046</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>리피파이가 애정으로 한 알 한 알 손수 뭉친 진주빛 알갱이 펄 파우더. 사역마에게 사용하면 체력을 5 회복시켜준다.</t>
+          <t>파우더 가루</t>
         </is>
       </c>
       <c r="C89" t="inlineStr"/>
@@ -1681,12 +1681,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000061</t>
+          <t>ItemData.Item.1000046.8</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>폭신폭신 사역마 쿠션</t>
+          <t>파우더 가루</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
@@ -1695,12 +1695,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000061.2</t>
+          <t>ItemData.Item.1000043</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>폭신폭신 사역마 쿠션</t>
+          <t>뽀송 프로그 데오도란트</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -1709,12 +1709,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000062</t>
+          <t>ItemData.Item.1000043.1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>보송송 목도리</t>
+          <t>이마에 맺힌 땀방울을 확실하게 잡아주는 뽀송 프로그 데오도란트. 기분 좋은 쿨링 효과가 체력을 50 회복시켜준다.</t>
         </is>
       </c>
       <c r="C92" t="inlineStr"/>
@@ -1723,12 +1723,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000062.3</t>
+          <t>ItemData.Item.1000044</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>추운 날씨엔 사역마에게 따스한 목도리를 둘러주자. 찬바람에 소모된 체력을 즉시 100 회복할 수 있다.</t>
+          <t>더스트 펄</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -1737,12 +1737,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000063</t>
+          <t>ItemData.Item.1000044.1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>실키 퍼프</t>
+          <t>리피파이가 애정으로 한 알 한 알 손수 뭉친 진주빛 알갱이 펄 파우더. 사역마에게 사용하면 체력을 5 회복시켜준다.</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -1751,12 +1751,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000063.1</t>
+          <t>ItemData.Item.1000061</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>지쳐서 푸석해진 사역마를 순식간에 뽀송하게 되돌려주는 실키 퍼프.</t>
+          <t>폭신폭신 사역마 쿠션</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -1765,12 +1765,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000045</t>
+          <t>ItemData.Item.1000061.2</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>노랑 파우더 가루</t>
+          <t>폭신폭신 사역마 쿠션</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -1779,12 +1779,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000045.1</t>
+          <t>ItemData.Item.1000062</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>미정</t>
+          <t>보송송 목도리</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -1793,12 +1793,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000064</t>
+          <t>ItemData.Item.1000062.3</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>솜솜가루</t>
+          <t>추운 날씨엔 사역마에게 따스한 목도리를 둘러주자. 찬바람에 소모된 체력을 즉시 100 회복할 수 있다.</t>
         </is>
       </c>
       <c r="C98" t="inlineStr"/>
@@ -1807,12 +1807,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000064.2</t>
+          <t>ItemData.Item.1000063</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>홈베이킹에 쓰이는 가정용 솜사탕 재료. 솜사탕 가게에서 조금씩 얻을 수 있다?</t>
+          <t>실키 퍼프</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -1821,12 +1821,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000065</t>
+          <t>ItemData.Item.1000063.1</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>솜솜 열매</t>
+          <t>지쳐서 푸석해진 사역마를 순식간에 뽀송하게 되돌려주는 실키 퍼프.</t>
         </is>
       </c>
       <c r="C100" t="inlineStr"/>
@@ -1835,12 +1835,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000065.3</t>
+          <t>ItemData.Item.1000045</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>달달한 솜이 폭신하게 열린 솜솜 열매. 잘 심어 가꾸면 더 많은 솜사탕 재료를 얻을 수 있을 것이다.</t>
+          <t>노랑 파우더 가루</t>
         </is>
       </c>
       <c r="C101" t="inlineStr"/>
@@ -1849,12 +1849,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000066</t>
+          <t>ItemData.Item.1000045.1</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>푸른 꿈결정</t>
+          <t>미정</t>
         </is>
       </c>
       <c r="C102" t="inlineStr"/>
@@ -1863,12 +1863,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000066.4</t>
+          <t>ItemData.Item.1000064</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>홈베이킹용 솜솜가루가 달빛을 지나치게 흡수해 파랗게 물든 꿈결정. 때로는 실패가 성공보다 더 아름다운 결과를 가져오는 법이다.</t>
+          <t>솜솜가루</t>
         </is>
       </c>
       <c r="C103" t="inlineStr"/>
@@ -1877,12 +1877,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000067</t>
+          <t>ItemData.Item.1000064.2</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>솜사타</t>
+          <t>홈베이킹에 쓰이는 가정용 솜사탕 재료. 솜사탕 가게에서 조금씩 얻을 수 있다?</t>
         </is>
       </c>
       <c r="C104" t="inlineStr"/>
@@ -1891,12 +1891,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000067.1</t>
+          <t>ItemData.Item.1000065</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>솜사타에 올라타! 바람처럼 빠르게 데려다줄거야!</t>
+          <t>솜솜 열매</t>
         </is>
       </c>
       <c r="C105" t="inlineStr"/>
@@ -1905,12 +1905,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000068</t>
+          <t>ItemData.Item.1000065.3</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>페로페로 향수</t>
+          <t>달달한 솜이 폭신하게 열린 솜솜 열매. 잘 심어 가꾸면 더 많은 솜사탕 재료를 얻을 수 있을 것이다.</t>
         </is>
       </c>
       <c r="C106" t="inlineStr"/>
@@ -1919,12 +1919,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000068.1</t>
+          <t>ItemData.Item.1000066</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>저항할 수 없는 묘한 향기를 풍겨 근처에 있는 사역마를 끌어당기는 미스테리한 향수. 매료된 사역마는 임시 계약을 맺어 하루 동안 당신을 돕는 데에 동의할 것이다.</t>
+          <t>푸른 꿈결정</t>
         </is>
       </c>
       <c r="C107" t="inlineStr"/>
@@ -1933,12 +1933,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000069</t>
+          <t>ItemData.Item.1000066.4</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>솜솜 보틀</t>
+          <t>홈베이킹용 솜솜가루가 달빛을 지나치게 흡수해 파랗게 물든 꿈결정. 때로는 실패가 성공보다 더 아름다운 결과를 가져오는 법이다.</t>
         </is>
       </c>
       <c r="C108" t="inlineStr"/>
@@ -1947,12 +1947,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ItemData.Item.1000069.1</t>
+          <t>ItemData.Item.1000067</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>달콤한 솜사탕을 집에서도 만들고 싶다면 솜솜 보틀이 필요할 것이다. 전용 용기가 솜사탕의 달콤함을 오래도록 지켜줄 테니까!</t>
+          <t>솜사타</t>
         </is>
       </c>
       <c r="C109" t="inlineStr"/>
@@ -1961,12 +1961,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000007</t>
+          <t>ItemData.Item.1000067.1</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>로딩 내용 어쩌고 저쩌고1</t>
+          <t>솜사타에 올라타! 바람처럼 빠르게 데려다줄거야!</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
@@ -1975,12 +1975,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000008</t>
+          <t>ItemData.Item.1000068</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>로딩 내용 어쩌고 저쩌고2</t>
+          <t>페로페로 향수</t>
         </is>
       </c>
       <c r="C111" t="inlineStr"/>
@@ -1989,12 +1989,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000027</t>
+          <t>ItemData.Item.1000068.1</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>솜사탕상점 로딩화면</t>
+          <t>저항할 수 없는 묘한 향기를 풍겨 근처에 있는 사역마를 끌어당기는 미스테리한 향수. 매료된 사역마는 임시 계약을 맺어 하루 동안 당신을 돕는 데에 동의할 것이다.</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
@@ -2003,12 +2003,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000028</t>
+          <t>ItemData.Item.1000069</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>파우더상점 로딩화면</t>
+          <t>솜솜 보틀</t>
         </is>
       </c>
       <c r="C113" t="inlineStr"/>
@@ -2017,12 +2017,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LoadingData.Loading.1000029</t>
+          <t>ItemData.Item.1000069.1</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>이불상점 로딩화면</t>
+          <t>달콤한 솜사탕을 집에서도 만들고 싶다면 솜솜 보틀이 필요할 것이다. 전용 용기가 솜사탕의 달콤함을 오래도록 지켜줄 테니까!</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -2031,12 +2031,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MapNpcData.MapNpcMenu.1000009.1</t>
+          <t>LoadingData.Loading.1000007</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>미니게임 시작</t>
+          <t>로딩 내용 어쩌고 저쩌고1</t>
         </is>
       </c>
       <c r="C115" t="inlineStr"/>
@@ -2045,12 +2045,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MapNpcData.MapNpcMenu.1000030.1</t>
+          <t>LoadingData.Loading.1000008</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>말걸기</t>
+          <t>로딩 내용 어쩌고 저쩌고2</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>MapNpcData.MapNpcMenu.1000078.1</t>
+          <t>LoadingData.Loading.1000027</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>말걸기</t>
+          <t>솜사탕상점 로딩화면</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -2073,12 +2073,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>MapNpcData.MapStaticNpcMenu.1000031.1</t>
+          <t>LoadingData.Loading.1000028</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>미니게임 시작</t>
+          <t>파우더상점 로딩화면</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
@@ -2087,16 +2087,86 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>MapNpcData.MapStaticNpcMenu.1000084.1</t>
+          <t>LoadingData.Loading.1000029</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>미니게임 시작</t>
+          <t>이불상점 로딩화면</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>MapNpcData.MapNpcMenu.1000009.1</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>미니게임 시작</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr"/>
+      <c r="D120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>MapNpcData.MapNpcMenu.1000030.1</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>말걸기</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr"/>
+      <c r="D121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>MapNpcData.MapNpcMenu.1000078.1</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>말걸기</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr"/>
+      <c r="D122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>MapNpcData.MapStaticNpcMenu.1000031.1</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>미니게임 시작</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr"/>
+      <c r="D123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>MapNpcData.MapStaticNpcMenu.1000084.1</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>미니게임 시작</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr"/>
+      <c r="D124" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>